<commit_message>
Class diary right after saving attendance; fix the Add student button on phones
- After attendance is saved, "Write class diary" opens the class note for the same date; a line explains it reaches every child who was not absent.
- The floating Add student button is a pill instead of an oval in pill-shaped looks, and the list leaves room so it no longer covers the last child.
- manual-qa: the diary cases now cover this path and check that an absent child does not get the class note (118 cases).
</commit_message>
<xml_diff>
--- a/manual-qa/Signal-School-Test-Cases.xlsx
+++ b/manual-qa/Signal-School-Test-Cases.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Summary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test cases'!$A$1:$M$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test cases'!$A$1:$M$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M117"/>
+  <dimension ref="A1:M119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Today → Class diary</t>
+          <t>Take attendance → Write class diary</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Tap "Class diary" on Std 1 A. Write a note and save.</t>
+          <t>Open Std 1 A attendance. Mark Aryan Mhatre "A" and tap "Save attendance". Under "Saved at…" tap "Write class diary". Write a note and save.</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -2120,12 +2120,12 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>"Diary saved". The note shows with today's date and "by Sunita Patil".</t>
+          <t>The diary form opens with the same date as the attendance. After Save: "Diary saved".</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Students</t>
+          <t>Teacher – Diary</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -2160,23 +2160,23 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Today → Students</t>
+          <t>Students → Riya Kale / Aryan Mhatre → Daily diary</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Tap "Students" on the Std 1 A card.</t>
+          <t>Open Riya Kale, then the "Daily diary" tab. Then do the same for Aryan Mhatre.</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>The Std 1 A class list opens with photos (or initials), roll numbers and today's mark.</t>
+          <t>Riya (not absent): the class note shows with today's date, "Whole class" and "by Sunita Patil". Aryan (absent today): the class note is NOT shown.</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Students</t>
+          <t>Teacher – Diary</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -2211,27 +2211,27 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Students → search</t>
+          <t>Today → Class diary</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Type in the search box.</t>
+          <t>Tap "Class diary" on the Std 1 A card. Write a note and save.</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Riya</t>
+          <t>We sang a poem.</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale appears (Std 1 A).</t>
+          <t>"Diary saved". The note also shows in Riya Kale's "Daily diary".</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -2266,22 +2266,18 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Students → search</t>
+          <t>Today → Students</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Search by the parent's mobile number.</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>9123400004</t>
-        </is>
-      </c>
+          <t>Tap "Students" on the Std 1 A card.</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr"/>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Kiran Thakur appears.</t>
+          <t>The Std 1 A class list opens with photos (or initials), roll numbers and today's mark.</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -2306,7 +2302,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Student profile</t>
+          <t>Teacher – Students</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -2321,18 +2317,22 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Students → Riya Kale</t>
+          <t>Students → search</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Open Riya Kale.</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr"/>
+          <t>Type in the search box.</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Riya</t>
+        </is>
+      </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Photo, "Std 1 A", Roll no., GR number, age, "Sunil Kale · Father" with call and WhatsApp icons, and tabs: Details, Daily diary, Past years, Report card, Health. "Attendance this month" shows a small calendar with totals.</t>
+          <t>Riya Kale appears (Std 1 A).</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Student profile</t>
+          <t>Teacher – Students</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -2372,18 +2372,22 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale → Past years</t>
+          <t>Students → search</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Open the "Past years" tab.</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr"/>
+          <t>Search by the parent's mobile number.</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>9123400004</t>
+        </is>
+      </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>Shows last year: Balwadi A, "Moved to next class", with that year's attendance.</t>
+          <t>Kiran Thakur appears.</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -2423,27 +2427,23 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale → Daily diary</t>
+          <t>Students → Riya Kale</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Add a note about the child and save.</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>Riya read a full story today.</t>
-        </is>
-      </c>
+          <t>Open Riya Kale.</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr"/>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>Note appears at the top with today's date and "by Sunita Patil".</t>
+          <t>Photo, "Std 1 A", Roll no., GR number, age, "Sunil Kale · Father" with call and WhatsApp icons, and tabs: Details, Daily diary, Past years, Report card, Health. "Attendance this month" shows a small calendar with totals.</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
@@ -2478,18 +2478,18 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale → call / WhatsApp</t>
+          <t>Riya Kale → Past years</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Tap the phone icon. Go back. Tap the WhatsApp icon.</t>
+          <t>Open the "Past years" tab.</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr"/>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Phone dialer opens with 9123400001. WhatsApp opens a chat to that number (if WhatsApp is installed).</t>
+          <t>Shows last year: Balwadi A, "Moved to next class", with that year's attendance.</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -2529,27 +2529,27 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Aryan Mhatre → camera icon</t>
+          <t>Riya Kale → Daily diary</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Open Aryan Mhatre (no photo). Tap the camera icon on the picture, choose the photo file.</t>
+          <t>Add a note about the child and save.</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>test-files/child-photo-boy.jpg</t>
+          <t>Riya read a full story today.</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>The photo shows on the profile and in the class list.</t>
+          <t>Note appears at the top with today's date and "by Sunita Patil".</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
@@ -2584,22 +2584,18 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Aryan Mhatre → camera icon</t>
+          <t>Riya Kale → call / WhatsApp</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Try to upload the wrong files as a photo.</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>not-a-photo.pdf, then photo-too-big-9MB.png</t>
-        </is>
-      </c>
+          <t>Tap the phone icon. Go back. Tap the WhatsApp icon.</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr"/>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>PDF: "This file type is not allowed" (or it cannot be picked). Big file: "The file is too large". The old photo stays.</t>
+          <t>Phone dialer opens with 9123400001. WhatsApp opens a chat to that number (if WhatsApp is installed).</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -2639,27 +2635,27 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale → Edit</t>
+          <t>Aryan Mhatre → camera icon</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Tap "Edit", change the address, tap "Save student".</t>
+          <t>Open Aryan Mhatre (no photo). Tap the camera icon on the picture, choose the photo file.</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>New address: Kopri, Thane</t>
+          <t>test-files/child-photo-boy.jpg</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>"Saved". Details tab shows the new address.</t>
+          <t>The photo shows on the profile and in the class list.</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
@@ -2694,22 +2690,22 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale → Health</t>
+          <t>Aryan Mhatre → camera icon</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Add a health check-up: today's date, height and weight. Save.</t>
+          <t>Try to upload the wrong files as a photo.</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Height 112, Weight 19</t>
+          <t>not-a-photo.pdf, then photo-too-big-9MB.png</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>The check-up shows in the list with "Height: 112 cm", "Weight: 19 kg".</t>
+          <t>PDF: "This file type is not allowed" (or it cannot be picked). Big file: "The file is too large". The old photo stays.</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
@@ -2734,7 +2730,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Students</t>
+          <t>Teacher – Student profile</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -2749,27 +2745,27 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Students → Add student</t>
+          <t>Riya Kale → Edit</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Tap "Add student". Fill name, class, gender. Tap "Save student".</t>
+          <t>Tap "Edit", change the address, tap "Save student".</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>QA Child One, Std 1 A, Girl</t>
+          <t>New address: Kopri, Thane</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>Message "QA Child One added with register number SS-…". The child is in the Std 1 A list.</t>
+          <t>"Saved". Details tab shows the new address.</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
@@ -2789,7 +2785,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Students</t>
+          <t>Teacher – Student profile</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -2804,27 +2800,27 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Students → Add student</t>
+          <t>Riya Kale → Health</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Add a child with the same name and parent mobile as an existing child.</t>
+          <t>Add a health check-up: today's date, height and weight. Save.</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale, Std 1 A, mobile 9123400001</t>
+          <t>Height 112, Weight 19</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>Question "Is this child already in the school records?" shows Riya Kale. Tap Cancel: nothing is added.</t>
+          <t>The check-up shows in the list with "Height: 112 cm", "Weight: 19 kg".</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
@@ -2844,7 +2840,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Syllabus</t>
+          <t>Teacher – Students</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2859,22 +2855,22 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Syllabus → Maths · Std 1 A</t>
+          <t>Students → Add student</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Open a subject. Tap "Mark as taught" on a topic that is not taught yet. Then undo with "Mark as not taught".</t>
+          <t>Tap "Add student". Fill name, class, gender. Tap "Save student".</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Maths · Std 1 A</t>
+          <t>QA Child One, Std 1 A, Girl</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>The topic shows "Taught on (today) by Me" and the % goes up; after undo it goes back.</t>
+          <t>Message "QA Child One added with register number SS-…". The child is in the Std 1 A list.</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -2899,7 +2895,7 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Marks</t>
+          <t>Teacher – Students</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -2914,22 +2910,22 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>More → Marks</t>
+          <t>Students → Add student</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Choose Class Std 1 A, Subject Maths, Term Semester 1. In "Maximum marks for everyone" type 50 and tap "Fill in". Enter marks for 3 children. Save.</t>
+          <t>Add a child with the same name and parent mobile as an existing child.</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Marks: 45, 30, 12</t>
+          <t>Riya Kale, Std 1 A, mobile 9123400001</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>"Saved". Reopen Marks: the numbers are still there.</t>
+          <t>Question "Is this child already in the school records?" shows Riya Kale. Tap Cancel: nothing is added.</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
@@ -2954,7 +2950,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Marks</t>
+          <t>Teacher – Syllabus</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -2969,27 +2965,27 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>More → Marks</t>
+          <t>Syllabus → Maths · Std 1 A</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Enter marks higher than "Out of".</t>
+          <t>Open a subject. Tap "Mark as taught" on a topic that is not taught yet. Then undo with "Mark as not taught".</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>60 out of 50</t>
+          <t>Maths · Std 1 A</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>Message "More than maximum marks". Not saved.</t>
+          <t>The topic shows "Taught on (today) by Me" and the % goes up; after undo it goes back.</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -3024,23 +3020,27 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale → Report card</t>
+          <t>More → Marks</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Open the "Report card" tab, choose Semester 1, tap "Open report card", then "Print / Save PDF".</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr"/>
+          <t>Choose Class Std 1 A, Subject Maths, Term Semester 1. In "Maximum marks for everyone" type 50 and tap "Fill in". Enter marks for 3 children. Save.</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Marks: 45, 30, 12</t>
+        </is>
+      </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>Shows school name, child details, marks, attendance line and signature lines (Class teacher, Principal, Parent). The print / save as PDF screen opens.</t>
+          <t>"Saved". Reopen Marks: the numbers are still there.</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Old year</t>
+          <t>Teacher – Marks</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -3075,18 +3075,22 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Year box at the top</t>
+          <t>More → Marks</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Change the year at the top from 2026-27 to the year before. Open Attendance and a child. Then choose the current year again.</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr"/>
+          <t>Enter marks higher than "Out of".</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>60 out of 50</t>
+        </is>
+      </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>Banner "You are viewing … Old years can be seen but not changed." Nothing can be saved in the old year. "Back to …" returns to the current year.</t>
+          <t>Message "More than maximum marks". Not saved.</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -3111,7 +3115,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Me</t>
+          <t>Teacher – Marks</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -3126,23 +3130,23 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>More → Me → Language</t>
+          <t>Riya Kale → Report card</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Choose हिंदी. Open Today, Attendance, Students. Then choose English again.</t>
+          <t>Open the "Report card" tab, choose Semester 1, tap "Open report card", then "Print / Save PDF".</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>The whole app (menus, buttons, messages) is in Hindi, then back to English. Note any word still in English.</t>
+          <t>Shows school name, child details, marks, attendance line and signature lines (Class teacher, Principal, Parent). The print / save as PDF screen opens.</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
@@ -3162,7 +3166,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Me</t>
+          <t>Teacher – Old year</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -3177,18 +3181,18 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>More → Me → Text size</t>
+          <t>Year box at the top</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Choose the biggest "Aa". Open Today and Take attendance. Then choose Normal again.</t>
+          <t>Change the year at the top from 2026-27 to the year before. Open Attendance and a child. Then choose the current year again.</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>Text gets bigger everywhere. Nothing overlaps or is cut, no sideways scrolling. Back to normal after.</t>
+          <t>Banner "You are viewing … Old years can be seen but not changed." Nothing can be saved in the old year. "Back to …" returns to the current year.</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
@@ -3228,27 +3232,23 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>More → Me → photo</t>
+          <t>More → Me → Language</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Tap the camera on your own picture and choose a photo.</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>test-files/teacher-photo.jpg</t>
-        </is>
-      </c>
+          <t>Choose हिंदी. Open Today, Attendance, Students. Then choose English again.</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>Your photo shows on the Me page.</t>
+          <t>The whole app (menus, buttons, messages) is in Hindi, then back to English. Note any word still in English.</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Access</t>
+          <t>Teacher – Me</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -3283,23 +3283,23 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Menus</t>
+          <t>More → Me → Text size</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Look at the menus. Then type /staff at the end of the app address and open it.</t>
+          <t>Choose the biggest "Aa". Open Today and Take attendance. Then choose Normal again.</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr"/>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>No "Teachers &amp; staff", "School settings", "Academic years" or "Activity log" for a teacher. Opening /staff goes back to the Today page.</t>
+          <t>Text gets bigger everywhere. Nothing overlaps or is cut, no sideways scrolling. Back to normal after.</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
@@ -3319,12 +3319,12 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Teacher – Subject teacher</t>
+          <t>Teacher – Me</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Teacher (Rahul)</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -3334,27 +3334,27 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>More → Me → photo</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Log in as Rahul.</t>
+          <t>Tap the camera on your own picture and choose a photo.</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>rahul@demo.test</t>
+          <t>test-files/teacher-photo.jpg</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>Std 5 A card shows attendance already done (green). "My subjects" lists Maths and English for Std 5 A, 6 A, 7 A.</t>
+          <t>Your photo shows on the Me page.</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
@@ -3369,42 +3369,38 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>CL-01</t>
+          <t>TC-37</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Office clerk</t>
+          <t>Teacher – Access</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Office clerk</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Menus</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Log in as the clerk.</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>clerk@demo.test</t>
-        </is>
-      </c>
+          <t>Look at the menus. Then type /staff at the end of the app address and open it.</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr"/>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>Opens the Dashboard. Menu has Dashboard, Attendance, Students, Syllabus, Me. No Marks and no school setup pages.</t>
+          <t>No "Teachers &amp; staff", "School settings", "Academic years" or "Activity log" for a teacher. Opening /staff goes back to the Today page.</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
@@ -3424,43 +3420,47 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>CL-02</t>
+          <t>TC-38</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Office clerk</t>
+          <t>Teacher – Subject teacher</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Office clerk</t>
+          <t>Teacher (Rahul)</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Attendance → Std 1 A</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Open Attendance, then a class.</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr"/>
+          <t>Log in as Rahul.</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>rahul@demo.test</t>
+        </is>
+      </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>The class list is shown with a note "You can see this attendance, but only teachers and the principal can change it." No Save button.</t>
+          <t>Std 5 A card shows attendance already done (green). "My subjects" lists Maths and English for Std 5 A, 6 A, 7 A.</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3475,7 +3475,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>CL-03</t>
+          <t>CL-01</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -3495,22 +3495,22 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Students → Add student</t>
+          <t>Menu</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Add a child with all details: open "More details (parents, address, documents)" and fill them. Leave "Register number (GR)" empty.</t>
+          <t>Log in as the clerk.</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>QA Child Two, Std 2 A, Boy, DOB 10/05/2019, parent Sunita Rane 9876501234, address Kalwa</t>
+          <t>clerk@demo.test</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>Saved with the next register number (SS-…). All details show on the profile.</t>
+          <t>Opens the Dashboard. Menu has Dashboard, Attendance, Students, Syllabus, Me. No Marks and no school setup pages.</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
@@ -3530,7 +3530,7 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>CL-04</t>
+          <t>CL-02</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
@@ -3550,27 +3550,23 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Students → Add student</t>
+          <t>Attendance → Std 1 A</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Tick "Date of birth not known" and fill approximate age.</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>QA Child Three, Std 3 A, age 8</t>
-        </is>
-      </c>
+          <t>Open Attendance, then a class.</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>Saved. The profile shows the age as approximate.</t>
+          <t>The class list is shown with a note "You can see this attendance, but only teachers and the principal can change it." No Save button.</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
@@ -3585,7 +3581,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>CL-05</t>
+          <t>CL-03</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
@@ -3610,22 +3606,22 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Type a wrong mobile number.</t>
+          <t>Add a child with all details: open "More details (parents, address, documents)" and fill them. Leave "Register number (GR)" empty.</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>12345</t>
+          <t>QA Child Two, Std 2 A, Boy, DOB 10/05/2019, parent Sunita Rane 9876501234, address Kalwa</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>Message "Enter a valid mobile number". Not saved until fixed.</t>
+          <t>Saved with the next register number (SS-…). All details show on the profile.</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -3640,12 +3636,12 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>CL-06</t>
+          <t>CL-04</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Import</t>
+          <t>Office clerk</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -3660,18 +3656,22 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Students → Import from Excel</t>
+          <t>Students → Add student</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Tap "Download template" and open the file.</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr"/>
+          <t>Tick "Date of birth not known" and fill approximate age.</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>QA Child Three, Std 3 A, age 8</t>
+        </is>
+      </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>An Excel file downloads with columns name*, class*, gender, date_of_birth … and a Help sheet listing the classes.</t>
+          <t>Saved. The profile shows the age as approximate.</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
@@ -3691,12 +3691,12 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>CL-07</t>
+          <t>CL-05</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Import</t>
+          <t>Office clerk</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -3711,27 +3711,27 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Students → Import from Excel</t>
+          <t>Students → Add student</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Choose the good file. Check the rows. Tap "Import 5 students".</t>
+          <t>Type a wrong mobile number.</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>test-files/students-import-5-good.xlsx</t>
+          <t>12345</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>"5 of 5 rows are ready". After import: "5 students imported". Asha Lokhande and Rohan Dhotre are now in Std 1 A.</t>
+          <t>Message "Enter a valid mobile number". Not saved until fixed.</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>CL-08</t>
+          <t>CL-06</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
@@ -3771,22 +3771,18 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Choose the file with mistakes.</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>test-files/students-import-with-errors.xlsx</t>
-        </is>
-      </c>
+          <t>Tap "Download template" and open the file.</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr"/>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>"1 of 5 rows are ready". Problems in red: Ajay Borse "Class: Class not found", row 4 "Full name: Required", Tara Jogdand "Date of birth: Wrong date (use DD/MM/YYYY)", Vikas Ingle "Parent mobile number: Please check this". "Import 1 student" adds only Meghna Salve.</t>
+          <t>An Excel file downloads with columns name*, class*, gender, date_of_birth … and a Help sheet listing the classes.</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
@@ -3801,7 +3797,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>CL-09</t>
+          <t>CL-07</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -3816,7 +3812,7 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -3826,22 +3822,22 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>On a phone, import the CSV file.</t>
+          <t>Choose the good file. Check the rows. Tap "Import 5 students".</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>test-files/students-import-3-rows.csv</t>
+          <t>test-files/students-import-5-good.xlsx</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>"3 of 3 rows are ready", then "3 students imported".</t>
+          <t>"5 of 5 rows are ready". After import: "5 students imported". Asha Lokhande and Rohan Dhotre are now in Std 1 A.</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
@@ -3856,7 +3852,7 @@
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>CL-10</t>
+          <t>CL-08</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
@@ -3881,22 +3877,22 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Choose the PDF file.</t>
+          <t>Choose the file with mistakes.</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>test-files/not-a-photo.pdf</t>
+          <t>test-files/students-import-with-errors.xlsx</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>"This file type is not allowed". Nothing imported.</t>
+          <t>"1 of 5 rows are ready". Problems in red: Ajay Borse "Class: Class not found", row 4 "Full name: Required", Tara Jogdand "Date of birth: Wrong date (use DD/MM/YYYY)", Vikas Ingle "Parent mobile number: Please check this". "Import 1 student" adds only Meghna Salve.</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
@@ -3911,12 +3907,12 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>CL-11</t>
+          <t>CL-09</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Leaving</t>
+          <t>Office clerk – Import</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -3926,32 +3922,32 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Nikhil Sonawane → Mark as left school</t>
+          <t>Students → Import from Excel</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Open Nikhil Sonawane. Tap "Mark as left school". Choose a reason, add a note, confirm.</t>
+          <t>On a phone, import the CSV file.</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Reason: Joined another school; note: Moved to TMC School No. 12</t>
+          <t>test-files/students-import-3-rows.csv</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>Status "Left school" with the date. Nikhil is no longer in the Std 3 A attendance list.</t>
+          <t>"3 of 3 rows are ready", then "3 students imported".</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
@@ -3966,12 +3962,12 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>CL-12</t>
+          <t>CL-10</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Leaving</t>
+          <t>Office clerk – Import</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -3981,28 +3977,32 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Nikhil Sonawane → Leaving certificate</t>
+          <t>Students → Import from Excel</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Tap "Leaving certificate", then "Print / Save PDF".</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr"/>
+          <t>Choose the PDF file.</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>test-files/not-a-photo.pdf</t>
+        </is>
+      </c>
       <c r="H62" s="5" t="inlineStr">
         <is>
-          <t>Certificate with school name, GR number, name, parents, date of birth, last class, attendance, date of leaving. Print / save as PDF opens; nothing is cut off.</t>
+          <t>"This file type is not allowed". Nothing imported.</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
@@ -4017,7 +4017,7 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>CL-13</t>
+          <t>CL-11</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -4032,28 +4032,32 @@
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Riya Kale → (address)/certificate</t>
+          <t>Nikhil Sonawane → Mark as left school</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Open Riya Kale, add /certificate at the end of the address.</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="inlineStr"/>
+          <t>Open Nikhil Sonawane. Tap "Mark as left school". Choose a reason, add a note, confirm.</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>Reason: Joined another school; note: Moved to TMC School No. 12</t>
+        </is>
+      </c>
       <c r="H63" s="5" t="inlineStr">
         <is>
-          <t>Message "This child is still studying here. Mark the child as left before printing the certificate."</t>
+          <t>Status "Left school" with the date. Nikhil is no longer in the Std 3 A attendance list.</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
@@ -4068,12 +4072,12 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>CL-14</t>
+          <t>CL-12</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Search</t>
+          <t>Office clerk – Leaving</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
@@ -4088,22 +4092,18 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>Students → search</t>
+          <t>Nikhil Sonawane → Leaving certificate</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Search "Lata". Then tick "Search all years".</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
-        <is>
-          <t>Lata</t>
-        </is>
-      </c>
+          <t>Tap "Leaving certificate", then "Print / Save PDF".</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr"/>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>Without the tick: "No students found". With the tick: Lata Bhalerao, "Left school".</t>
+          <t>Certificate with school name, GR number, name, parents, date of birth, last class, attendance, date of leaving. Print / save as PDF opens; nothing is cut off.</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
@@ -4123,12 +4123,12 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>CL-15</t>
+          <t>CL-13</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Search</t>
+          <t>Office clerk – Leaving</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -4138,32 +4138,28 @@
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Lata Bhalerao → Re-admit</t>
+          <t>Riya Kale → (address)/certificate</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Open Lata. Tap "Re-admit", choose Std 3 A, confirm.</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr">
-        <is>
-          <t>Std 3 A</t>
-        </is>
-      </c>
+          <t>Open Riya Kale, add /certificate at the end of the address.</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr"/>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>"Saved". Lata is "Studying" in Std 3 A and appears in Std 3 A attendance. Her old year stays under "Past years".</t>
+          <t>Message "This child is still studying here. Mark the child as left before printing the certificate."</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
@@ -4178,12 +4174,12 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>CL-16</t>
+          <t>CL-14</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Health</t>
+          <t>Office clerk – Search</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -4198,23 +4194,27 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Swati Gholap → Health</t>
+          <t>Students → search</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Open Swati Gholap, tab Health.</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr"/>
+          <t>Search "Lata". Then tick "Search all years".</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Lata</t>
+        </is>
+      </c>
       <c r="H66" s="5" t="inlineStr">
         <is>
-          <t>Message "The last check-up says this child needs to see a doctor again." with the note about her eyes.</t>
+          <t>Without the tick: "No students found". With the tick: Lata Bhalerao, "Left school".</t>
         </is>
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
@@ -4229,12 +4229,12 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>CL-17</t>
+          <t>CL-15</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Students</t>
+          <t>Office clerk – Search</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
@@ -4244,28 +4244,32 @@
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Students → filters</t>
+          <t>Lata Bhalerao → Re-admit</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Use the Class filter (Std 4 A), then Status "Left school", then "All".</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="inlineStr"/>
+          <t>Open Lata. Tap "Re-admit", choose Std 3 A, confirm.</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>Std 3 A</t>
+        </is>
+      </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>The list and the count ("… children") change with each filter.</t>
+          <t>"Saved". Lata is "Studying" in Std 3 A and appears in Std 3 A attendance. Her old year stays under "Past years".</t>
         </is>
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J67" s="5" t="inlineStr">
@@ -4280,12 +4284,12 @@
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>CL-18</t>
+          <t>CL-16</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Students</t>
+          <t>Office clerk – Health</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -4295,28 +4299,28 @@
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Students → Download Excel</t>
+          <t>Swati Gholap → Health</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Tap "Download Excel".</t>
+          <t>Open Swati Gholap, tab Health.</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
       <c r="H68" s="5" t="inlineStr">
         <is>
-          <t>An Excel file with the children of the list downloads and opens.</t>
+          <t>Message "The last check-up says this child needs to see a doctor again." with the note about her eyes.</t>
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
@@ -4331,12 +4335,12 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>CL-19</t>
+          <t>CL-17</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Office clerk – Register</t>
+          <t>Office clerk – Students</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
@@ -4351,18 +4355,18 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Attendance → Monthly register</t>
+          <t>Students → filters</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Choose Std 1 A and this month. Tap "Download Excel", then "Print / Save PDF".</t>
+          <t>Use the Class filter (Std 4 A), then Status "Left school", then "All".</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr"/>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>Grid of children × days with P / A / L / LT, grey holidays, "Present each day" row. Excel downloads; print shows the whole register.</t>
+          <t>The list and the count ("… children") change with each filter.</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
@@ -4382,47 +4386,43 @@
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>PR-01</t>
+          <t>CL-18</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Principal – Dashboard</t>
+          <t>Office clerk – Students</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Office clerk</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Students → Download Excel</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Log in as the principal.</t>
-        </is>
-      </c>
-      <c r="G70" s="5" t="inlineStr">
-        <is>
-          <t>principal@demo.test</t>
-        </is>
-      </c>
+          <t>Tap "Download Excel".</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr"/>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>Dashboard with boxes: Students, Teachers, Classes, Attendance done today (x/8), Absent today, Meals to serve today. Numbers are not empty.</t>
+          <t>An Excel file with the children of the list downloads and opens.</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
@@ -4437,43 +4437,43 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>PR-02</t>
+          <t>CL-19</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Principal – Dashboard</t>
+          <t>Office clerk – Register</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Office clerk</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Attendance → Monthly register</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Look at "Attendance not taken".</t>
+          <t>Choose Std 1 A and this month. Tap "Download Excel", then "Print / Save PDF".</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr"/>
       <c r="H71" s="5" t="inlineStr">
         <is>
-          <t>Lists classes still waiting today (at the start: Std 1 A and Std 3 A). After a teacher saves, that class goes away.</t>
+          <t>Grid of children × days with P / A / L / LT, grey holidays, "Present each day" row. Excel downloads; print shows the whole register.</t>
         </is>
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
@@ -4488,7 +4488,7 @@
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>PR-03</t>
+          <t>PR-01</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
@@ -4503,27 +4503,27 @@
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>Dashboard → Absent several days in a row</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Find Kiran Thakur. Tap her WhatsApp icon.</t>
+          <t>Log in as the principal.</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>Kiran Thakur</t>
+          <t>principal@demo.test</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
         <is>
-          <t>Kiran Thakur, Std 4 A, "5 days". WhatsApp opens with a ready message to the family.</t>
+          <t>Dashboard with boxes: Students, Teachers, Classes, Attendance done today (x/8), Absent today, Meals to serve today. Numbers are not empty.</t>
         </is>
       </c>
       <c r="I72" s="5" t="inlineStr">
@@ -4543,7 +4543,7 @@
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>PR-04</t>
+          <t>PR-02</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -4563,23 +4563,23 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>Dashboard → Children who often miss school</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Look at the list.</t>
+          <t>Look at "Attendance not taken".</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr"/>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>Kiran Thakur is listed with her % (below 75%) and Std 4 A.</t>
+          <t>Lists classes still waiting today (at the start: Std 1 A and Std 3 A). After a teacher saves, that class goes away.</t>
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J73" s="5" t="inlineStr">
@@ -4594,7 +4594,7 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>PR-05</t>
+          <t>PR-03</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
@@ -4609,28 +4609,32 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>Dashboard (bottom)</t>
+          <t>Dashboard → Absent several days in a row</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>Scroll down.</t>
-        </is>
-      </c>
-      <c r="G74" s="5" t="inlineStr"/>
+          <t>Find Kiran Thakur. Tap her WhatsApp icon.</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>Kiran Thakur</t>
+        </is>
+      </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t>"Birthdays today: Ishaan Jagtap (Std 2 A)". Also "Attendance in the last 2 weeks" bars and "Syllabus progress" per class.</t>
+          <t>Kiran Thakur, Std 4 A, "5 days". WhatsApp opens with a ready message to the family.</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
@@ -4645,7 +4649,7 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>PR-06</t>
+          <t>PR-04</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
@@ -4665,23 +4669,23 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard → Children who often miss school</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>Look for the health box.</t>
+          <t>Look at the list.</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr"/>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>"… children need to see a doctor again (from the last health camp)".</t>
+          <t>Kiran Thakur is listed with her % (below 75%) and Std 4 A.</t>
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
@@ -4696,12 +4700,12 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>PR-07</t>
+          <t>PR-05</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Principal – Attendance</t>
+          <t>Principal – Dashboard</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
@@ -4716,23 +4720,23 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>Attendance</t>
+          <t>Dashboard (bottom)</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Open Attendance. Tap a class that is done. Change one mark and save.</t>
+          <t>Scroll down.</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr"/>
       <c r="H76" s="5" t="inlineStr">
         <is>
-          <t>Classes show "x present · y absent" or "Not done". The principal can change and save.</t>
+          <t>"Birthdays today: Ishaan Jagtap (Std 2 A)". Also "Attendance in the last 2 weeks" bars and "Syllabus progress" per class.</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
@@ -4747,12 +4751,12 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>PR-08</t>
+          <t>PR-06</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Principal – Attendance</t>
+          <t>Principal – Dashboard</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
@@ -4767,27 +4771,23 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>Attendance → class → Date</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Pick a date 10 days ago and change one mark. Save.</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
-        <is>
-          <t>10 days ago</t>
-        </is>
-      </c>
+          <t>Look for the health box.</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr"/>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>Saved (the principal may correct old days; a teacher may not).</t>
+          <t>"… children need to see a doctor again (from the last health camp)".</t>
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J77" s="5" t="inlineStr">
@@ -4802,12 +4802,12 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>PR-09</t>
+          <t>PR-07</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Principal – Staff</t>
+          <t>Principal – Attendance</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -4817,27 +4817,23 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>More → Teachers &amp; staff → Add teacher or staff</t>
+          <t>Attendance</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Add a new teacher.</t>
-        </is>
-      </c>
-      <c r="G78" s="5" t="inlineStr">
-        <is>
-          <t>Name: QA Teacher Two; Mobile 9820000099; Role Teacher</t>
-        </is>
-      </c>
+          <t>Open Attendance. Tap a class that is done. Change one mark and save.</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr"/>
       <c r="H78" s="5" t="inlineStr">
         <is>
-          <t>Box "Login details" with a temporary password. "Copy message for WhatsApp" → "Copied…". The teacher is in the Active list.</t>
+          <t>Classes show "x present · y absent" or "Not done". The principal can change and save.</t>
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
@@ -4857,12 +4853,12 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>PR-10</t>
+          <t>PR-08</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Principal – Staff</t>
+          <t>Principal – Attendance</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
@@ -4872,27 +4868,27 @@
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Teachers &amp; staff → Add</t>
+          <t>Attendance → class → Date</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Try to add someone with a mobile number already used.</t>
+          <t>Pick a date 10 days ago and change one mark. Save.</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>Mobile 9820000004</t>
+          <t>10 days ago</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>Not added: message "This already exists" (or "Already used" under the box).</t>
+          <t>Saved (the principal may correct old days; a teacher may not).</t>
         </is>
       </c>
       <c r="I79" s="5" t="inlineStr">
@@ -4912,7 +4908,7 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>PR-11</t>
+          <t>PR-09</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
@@ -4932,22 +4928,22 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>Teachers &amp; staff → Neha Joshi → Classes</t>
+          <t>More → Teachers &amp; staff → Add teacher or staff</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Open Neha Joshi, tab "Classes". Add: Std 2 A, Subject teacher, subject English. Then log in as Neha.</t>
+          <t>Add a new teacher.</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>newteacher@demo.test / NehaQa@2026</t>
+          <t>Name: QA Teacher Two; Mobile 9820000099; Role Teacher</t>
         </is>
       </c>
       <c r="H80" s="5" t="inlineStr">
         <is>
-          <t>The class shows in her list. Neha's Today page now shows "English · Std 2 A" under My subjects.</t>
+          <t>Box "Login details" with a temporary password. "Copy message for WhatsApp" → "Copied…". The teacher is in the Active list.</t>
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
@@ -4967,7 +4963,7 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>PR-12</t>
+          <t>PR-10</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -4987,23 +4983,27 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>Neha Joshi → Reset password</t>
+          <t>Teachers &amp; staff → Add</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>Tap "Reset password" and confirm. Log in as Neha with the new temporary password.</t>
-        </is>
-      </c>
-      <c r="G81" s="5" t="inlineStr"/>
+          <t>Try to add someone with a mobile number already used.</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>Mobile 9820000004</t>
+        </is>
+      </c>
       <c r="H81" s="5" t="inlineStr">
         <is>
-          <t>A new temporary password is shown once. Neha's old password stops working; with the new one she must choose her own password again.</t>
+          <t>Not added: message "This already exists" (or "Already used" under the box).</t>
         </is>
       </c>
       <c r="I81" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J81" s="5" t="inlineStr">
@@ -5018,7 +5018,7 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>PR-13</t>
+          <t>PR-11</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
@@ -5038,23 +5038,27 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>QA Teacher Two → Make inactive</t>
+          <t>Teachers &amp; staff → Neha Joshi → Classes</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>Tap "Make inactive" and confirm. Try to log in as that teacher. Then "Make active again".</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="inlineStr"/>
+          <t>Open Neha Joshi, tab "Classes". Add: Std 2 A, Subject teacher, subject English. Then log in as Neha.</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>newteacher@demo.test / NehaQa@2026</t>
+        </is>
+      </c>
       <c r="H82" s="5" t="inlineStr">
         <is>
-          <t>Teacher moves to the "Inactive" tab and cannot log in ("This account is inactive…"). After "Make active again" login works.</t>
+          <t>The class shows in her list. Neha's Today page now shows "English · Std 2 A" under My subjects.</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
@@ -5069,12 +5073,12 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>PR-14</t>
+          <t>PR-12</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Principal – Classes</t>
+          <t>Principal – Staff</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
@@ -5089,27 +5093,23 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>More → Classes &amp; subjects</t>
+          <t>Neha Joshi → Reset password</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>In Std 4 A type "Computer" in "New subject" and tap Add. Then remove it (x) and confirm.</t>
-        </is>
-      </c>
-      <c r="G83" s="5" t="inlineStr">
-        <is>
-          <t>Computer</t>
-        </is>
-      </c>
+          <t>Tap "Reset password" and confirm. Log in as Neha with the new temporary password.</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr"/>
       <c r="H83" s="5" t="inlineStr">
         <is>
-          <t>The subject appears as a chip and then is removed.</t>
+          <t>A new temporary password is shown once. Neha's old password stops working; with the new one she must choose her own password again.</t>
         </is>
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J83" s="5" t="inlineStr">
@@ -5124,12 +5124,12 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>PR-15</t>
+          <t>PR-13</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Principal – Classes</t>
+          <t>Principal – Staff</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -5144,23 +5144,23 @@
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>Classes &amp; subjects → Class levels</t>
+          <t>QA Teacher Two → Make inactive</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>Open "Class levels".</t>
+          <t>Tap "Make inactive" and confirm. Try to log in as that teacher. Then "Make active again".</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr"/>
       <c r="H84" s="5" t="inlineStr">
         <is>
-          <t>Levels Balwadi to Std 7 with their "Next class level"; Std 7 is "Last class of the school".</t>
+          <t>Teacher moves to the "Inactive" tab and cannot log in ("This account is inactive…"). After "Make active again" login works.</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr">
@@ -5175,7 +5175,7 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>PR-16</t>
+          <t>PR-14</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -5195,27 +5195,27 @@
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>Classes &amp; subjects → Activities</t>
+          <t>More → Classes &amp; subjects</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>Add a new activity. Open its members, tick 2 children and save.</t>
+          <t>In Std 4 A type "Computer" in "New subject" and tap Add. Then remove it (x) and confirm.</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>Chess club; Kiran Thakur, Riya Kale</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr">
         <is>
-          <t>The activity shows "2 members".</t>
+          <t>The subject appears as a chip and then is removed.</t>
         </is>
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J85" s="5" t="inlineStr">
@@ -5230,12 +5230,12 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>PR-17</t>
+          <t>PR-15</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Principal – Syllabus</t>
+          <t>Principal – Classes</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -5250,27 +5250,23 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>Syllabus → a subject → Edit chapters</t>
+          <t>Classes &amp; subjects → Class levels</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>Add a chapter, paste 3 topics (one per line), tap "Add these topics". Remove one new topic. Try to remove a topic that is already taught.</t>
-        </is>
-      </c>
-      <c r="G86" s="5" t="inlineStr">
-        <is>
-          <t>QA Chapter; Topic A / Topic B / Topic C</t>
-        </is>
-      </c>
+          <t>Open "Class levels".</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr"/>
       <c r="H86" s="5" t="inlineStr">
         <is>
-          <t>Chapter with 3 topics appears; removing a new topic works; a taught topic cannot be removed ("Already taught, so it cannot be removed").</t>
+          <t>Levels Balwadi to Std 7 with their "Next class level"; Std 7 is "Last class of the school".</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J86" s="5" t="inlineStr">
@@ -5285,12 +5281,12 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>PR-18</t>
+          <t>PR-16</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Principal – Holidays</t>
+          <t>Principal – Classes</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
@@ -5305,27 +5301,27 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>More → Holidays</t>
+          <t>Classes &amp; subjects → Activities</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Add a holiday for a date next week. Then delete it.</t>
+          <t>Add a new activity. Open its members, tick 2 children and save.</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>QA Holiday, next week, type Holiday</t>
+          <t>Chess club; Kiran Thakur, Riya Kale</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr">
         <is>
-          <t>Holiday shows in the list, then is removed. (Do NOT add a holiday for today.)</t>
+          <t>The activity shows "2 members".</t>
         </is>
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J87" s="5" t="inlineStr">
@@ -5340,12 +5336,12 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>PR-19</t>
+          <t>PR-17</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Principal – Years</t>
+          <t>Principal – Syllabus</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
@@ -5360,18 +5356,22 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>More → Academic years</t>
+          <t>Syllabus → a subject → Edit chapters</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>Look at the list.</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr"/>
+          <t>Add a chapter, paste 3 topics (one per line), tap "Add these topics". Remove one new topic. Try to remove a topic that is already taught.</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>QA Chapter; Topic A / Topic B / Topic C</t>
+        </is>
+      </c>
       <c r="H88" s="5" t="inlineStr">
         <is>
-          <t>2026-27 "Current", older years "Closed", each with dates, classes and number of students (not 0).</t>
+          <t>Chapter with 3 topics appears; removing a new topic works; a taught topic cannot be removed ("Already taught, so it cannot be removed").</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
@@ -5391,12 +5391,12 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>PR-20</t>
+          <t>PR-18</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Principal – Years</t>
+          <t>Principal – Holidays</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -5411,27 +5411,27 @@
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>Academic years → Start new academic year</t>
+          <t>More → Holidays</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Go through all 5 steps for 2027-28. On the last step keep "Make it current now" OFF. Tap "Create the new year".</t>
+          <t>Add a holiday for a date next week. Then delete it.</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>2027-28</t>
+          <t>QA Holiday, next week, type Holiday</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr">
         <is>
-          <t>"2027-28 is ready" with counts. The list shows 2027-28 as "Planned". IMPORTANT: do NOT make it current.</t>
+          <t>Holiday shows in the list, then is removed. (Do NOT add a holiday for today.)</t>
         </is>
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J89" s="5" t="inlineStr">
@@ -5446,7 +5446,7 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>PR-21</t>
+          <t>PR-19</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -5466,27 +5466,23 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>Academic years → (closed year) → Unlock for corrections</t>
+          <t>More → Academic years</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Unlock the last closed year for 10 minutes with a reason.</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>10 minutes; reason: QA test</t>
-        </is>
-      </c>
+          <t>Look at the list.</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr"/>
       <c r="H90" s="5" t="inlineStr">
         <is>
-          <t>"Unlocked until (time)". The activity log shows "Unlocked a year".</t>
+          <t>2026-27 "Current", older years "Closed", each with dates, classes and number of students (not 0).</t>
         </is>
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
@@ -5501,12 +5497,12 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>PR-22</t>
+          <t>PR-20</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>Principal – School</t>
+          <t>Principal – Years</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
@@ -5521,27 +5517,27 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>More → School settings → This school</t>
+          <t>Academic years → Start new academic year</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>Change the phone number and save. Tap "Upload school logo" and choose the logo.</t>
+          <t>Go through all 5 steps for 2027-28. On the last step keep "Make it current now" OFF. Tap "Create the new year".</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>Phone 022 2500 0099; test-files/school-logo.png</t>
+          <t>2027-28</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
-          <t>"Saved". The new logo appears at the top left of the app.</t>
+          <t>"2027-28 is ready" with counts. The list shows 2027-28 as "Planned". IMPORTANT: do NOT make it current.</t>
         </is>
       </c>
       <c r="I91" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J91" s="5" t="inlineStr">
@@ -5556,12 +5552,12 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>PR-23</t>
+          <t>PR-21</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Principal – School</t>
+          <t>Principal – Years</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
@@ -5576,18 +5572,22 @@
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>School settings → This school</t>
+          <t>Academic years → (closed year) → Unlock for corrections</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Look at "Register number prefix" and "Days teachers can change old attendance".</t>
-        </is>
-      </c>
-      <c r="G92" s="5" t="inlineStr"/>
+          <t>Unlock the last closed year for 10 minutes with a reason.</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>10 minutes; reason: QA test</t>
+        </is>
+      </c>
       <c r="H92" s="5" t="inlineStr">
         <is>
-          <t>Help text shows the next register number (e.g. "Next register number will be SS-…"). Do not change weekly holidays.</t>
+          <t>"Unlocked until (time)". The activity log shows "Unlocked a year".</t>
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
@@ -5607,12 +5607,12 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>PR-24</t>
+          <t>PR-22</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>Principal – Activity log</t>
+          <t>Principal – School</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
@@ -5627,18 +5627,22 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>More → Activity log</t>
+          <t>More → School settings → This school</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>Filter Person = Sunita Patil, then Kind of change = Attendance. Use "Older" / "Newer".</t>
-        </is>
-      </c>
-      <c r="G93" s="5" t="inlineStr"/>
+          <t>Change the phone number and save. Tap "Upload school logo" and choose the logo.</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>Phone 022 2500 0099; test-files/school-logo.png</t>
+        </is>
+      </c>
       <c r="H93" s="5" t="inlineStr">
         <is>
-          <t>Shows who changed what and when, e.g. "Sunita Patil · Saved attendance · Std 1 A". Filters and pages work.</t>
+          <t>"Saved". The new logo appears at the top left of the app.</t>
         </is>
       </c>
       <c r="I93" s="5" t="inlineStr">
@@ -5658,12 +5662,12 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>PR-25</t>
+          <t>PR-23</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Principal – Phone</t>
+          <t>Principal – School</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
@@ -5673,28 +5677,28 @@
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>All pages on a phone</t>
+          <t>School settings → This school</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>On a phone, open every page from the bottom bar and "More".</t>
+          <t>Look at "Register number prefix" and "Days teachers can change old attendance".</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr"/>
       <c r="H94" s="5" t="inlineStr">
         <is>
-          <t>Every page fits the screen (no sideways scroll), all buttons can be tapped, nothing is hidden behind the bottom bar.</t>
+          <t>Help text shows the next register number (e.g. "Next register number will be SS-…"). Do not change weekly holidays.</t>
         </is>
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J94" s="5" t="inlineStr">
@@ -5709,47 +5713,43 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>OW-01</t>
+          <t>PR-24</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Trust owner</t>
+          <t>Principal – Activity log</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Trust owner</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>Me → School (or the school name)</t>
+          <t>More → Activity log</t>
         </is>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Switch to "Signal Shala, Nerul". Then switch back to Thane.</t>
-        </is>
-      </c>
-      <c r="G95" s="5" t="inlineStr">
-        <is>
-          <t>owner@demo.test</t>
-        </is>
-      </c>
+          <t>Filter Person = Sunita Patil, then Kind of change = Attendance. Use "Older" / "Newer".</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr"/>
       <c r="H95" s="5" t="inlineStr">
         <is>
-          <t>Nerul data is shown and the app colours change to the Marigold look; back in Thane the red Signal Shala look returns.</t>
+          <t>Shows who changed what and when, e.g. "Sunita Patil · Saved attendance · Std 1 A". Filters and pages work.</t>
         </is>
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J95" s="5" t="inlineStr">
@@ -5764,47 +5764,43 @@
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>OW-02</t>
+          <t>PR-25</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>Trust owner</t>
+          <t>Principal – Phone</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Trust owner</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>School settings → All schools</t>
+          <t>All pages on a phone</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Look at the table. Add a school.</t>
-        </is>
-      </c>
-      <c r="G96" s="5" t="inlineStr">
-        <is>
-          <t>QA School, Kalyan</t>
-        </is>
-      </c>
+          <t>On a phone, open every page from the bottom bar and "More".</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr"/>
       <c r="H96" s="5" t="inlineStr">
         <is>
-          <t>Both schools with students, teachers and attendance. The new school is added to the table.</t>
+          <t>Every page fits the screen (no sideways scroll), all buttons can be tapped, nothing is hidden behind the bottom bar.</t>
         </is>
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J96" s="5" t="inlineStr">
@@ -5819,47 +5815,47 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>OW-03</t>
+          <t>OW-01</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>Trust owner – second school</t>
+          <t>Trust owner</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Teacher (2nd school)</t>
+          <t>Trust owner</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>Me → School (or the school name)</t>
         </is>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>Log in as Imran.</t>
+          <t>Switch to "Signal Shala, Nerul". Then switch back to Thane.</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>imran@demo.test</t>
+          <t>owner@demo.test</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr">
         <is>
-          <t>Only Signal Shala, Nerul is shown, in the Marigold look. Thane children are not visible.</t>
+          <t>Nerul data is shown and the app colours change to the Marigold look; back in Thane the red Signal Shala look returns.</t>
         </is>
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J97" s="5" t="inlineStr">
@@ -5874,43 +5870,47 @@
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>LK-01</t>
+          <t>OW-02</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>Looks</t>
+          <t>Trust owner</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Trust owner</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Computer</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>More → School settings → Look</t>
+          <t>School settings → All schools</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>Open the Look tab.</t>
-        </is>
-      </c>
-      <c r="G98" s="5" t="inlineStr"/>
+          <t>Look at the table. Add a school.</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>QA School, Kalyan</t>
+        </is>
+      </c>
       <c r="H98" s="5" t="inlineStr">
         <is>
-          <t>6 looks with a small preview each: Signal Shala (In use), Blackboard, Notebook, Marigold, Calm teal, Easy to read.</t>
+          <t>Both schools with students, teachers and attendance. The new school is added to the table.</t>
         </is>
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J98" s="5" t="inlineStr">
@@ -5925,43 +5925,47 @@
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>LK-02</t>
+          <t>OW-03</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Looks</t>
+          <t>Trust owner – second school</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Teacher (2nd school)</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>School settings → Look</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Tap "Blackboard". Look around. Tap "Cancel".</t>
-        </is>
-      </c>
-      <c r="G99" s="5" t="inlineStr"/>
+          <t>Log in as Imran.</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>imran@demo.test</t>
+        </is>
+      </c>
       <c r="H99" s="5" t="inlineStr">
         <is>
-          <t>"You are trying “Blackboard”. Only you can see it." Colours, letters and icons change at once. Cancel returns to Signal Shala.</t>
+          <t>Only Signal Shala, Nerul is shown, in the Marigold look. Thane children are not visible.</t>
         </is>
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J99" s="5" t="inlineStr">
@@ -5976,7 +5980,7 @@
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>LK-03</t>
+          <t>LK-01</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
@@ -5986,7 +5990,7 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Principal + Teacher</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
@@ -5996,22 +6000,18 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t>School settings → Look</t>
+          <t>More → School settings → Look</t>
         </is>
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>Tap "Notebook", then "Use for the whole school". On another phone, log in (or reload) as Sunita.</t>
-        </is>
-      </c>
-      <c r="G100" s="5" t="inlineStr">
-        <is>
-          <t>sunita@demo.test</t>
-        </is>
-      </c>
+          <t>Open the Look tab.</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr"/>
       <c r="H100" s="5" t="inlineStr">
         <is>
-          <t>"Everyone in the school now sees “Notebook”". Sunita's app is in the Notebook look too.</t>
+          <t>6 looks with a small preview each: Signal Shala (In use), Blackboard, Notebook, Marigold, Calm teal, Easy to read.</t>
         </is>
       </c>
       <c r="I100" s="5" t="inlineStr">
@@ -6031,7 +6031,7 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>LK-04</t>
+          <t>LK-02</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -6051,18 +6051,18 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>Look: Signal Shala</t>
+          <t>School settings → Look</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>Use this look for the school. Open Today, Take attendance, Students, a student, Dashboard (as principal) on a phone.</t>
+          <t>Tap "Blackboard". Look around. Tap "Cancel".</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr"/>
       <c r="H101" s="5" t="inlineStr">
         <is>
-          <t>Red/white look with the traffic-light stripe. All text readable, buttons clear, icons match, nothing overlaps.</t>
+          <t>"You are trying “Blackboard”. Only you can see it." Colours, letters and icons change at once. Cancel returns to Signal Shala.</t>
         </is>
       </c>
       <c r="I101" s="5" t="inlineStr">
@@ -6082,7 +6082,7 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>LK-05</t>
+          <t>LK-03</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
@@ -6092,7 +6092,7 @@
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Principal + Teacher</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
@@ -6102,23 +6102,27 @@
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>Look: Blackboard</t>
+          <t>School settings → Look</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>Same pages as above.</t>
-        </is>
-      </c>
-      <c r="G102" s="5" t="inlineStr"/>
+          <t>Tap "Notebook", then "Use for the whole school". On another phone, log in (or reload) as Sunita.</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>sunita@demo.test</t>
+        </is>
+      </c>
       <c r="H102" s="5" t="inlineStr">
         <is>
-          <t>Green-board look with chalk-yellow and handwritten headings. Everything readable, no overlap.</t>
+          <t>"Everyone in the school now sees “Notebook”". Sunita's app is in the Notebook look too.</t>
         </is>
       </c>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J102" s="5" t="inlineStr">
@@ -6133,7 +6137,7 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>LK-06</t>
+          <t>LK-04</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
@@ -6153,23 +6157,23 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>Look: Notebook</t>
+          <t>Look: Signal Shala</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>Same pages as above.</t>
+          <t>Use this look for the school. Open Today, Take attendance, Students, a student, Dashboard (as principal) on a phone.</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr"/>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>Blue ink, ruled-page cards, sharp corners. Everything readable, no overlap.</t>
+          <t>Red/white look with the traffic-light stripe. All text readable, buttons clear, icons match, nothing overlaps.</t>
         </is>
       </c>
       <c r="I103" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J103" s="5" t="inlineStr">
@@ -6184,7 +6188,7 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>LK-07</t>
+          <t>LK-05</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
@@ -6204,7 +6208,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>Look: Marigold</t>
+          <t>Look: Blackboard</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
@@ -6215,7 +6219,7 @@
       <c r="G104" s="5" t="inlineStr"/>
       <c r="H104" s="5" t="inlineStr">
         <is>
-          <t>Saffron and maroon, soft round shapes. Everything readable, no overlap.</t>
+          <t>Green-board look with chalk-yellow and handwritten headings. Everything readable, no overlap.</t>
         </is>
       </c>
       <c r="I104" s="5" t="inlineStr">
@@ -6235,7 +6239,7 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>LK-08</t>
+          <t>LK-06</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -6255,7 +6259,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>Look: Calm teal</t>
+          <t>Look: Notebook</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
@@ -6266,7 +6270,7 @@
       <c r="G105" s="5" t="inlineStr"/>
       <c r="H105" s="5" t="inlineStr">
         <is>
-          <t>Teal and white, simple. Everything readable, no overlap.</t>
+          <t>Blue ink, ruled-page cards, sharp corners. Everything readable, no overlap.</t>
         </is>
       </c>
       <c r="I105" s="5" t="inlineStr">
@@ -6286,7 +6290,7 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>LK-09</t>
+          <t>LK-07</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
@@ -6306,18 +6310,18 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>Look: Easy to read</t>
+          <t>Look: Marigold</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>Same pages as above, also outside in sunlight if possible.</t>
+          <t>Same pages as above.</t>
         </is>
       </c>
       <c r="G106" s="5" t="inlineStr"/>
       <c r="H106" s="5" t="inlineStr">
         <is>
-          <t>Black on white, thick borders, bigger letters. Very easy to read.</t>
+          <t>Saffron and maroon, soft round shapes. Everything readable, no overlap.</t>
         </is>
       </c>
       <c r="I106" s="5" t="inlineStr">
@@ -6337,7 +6341,7 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>LK-10</t>
+          <t>LK-08</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -6347,28 +6351,28 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>More → Me</t>
+          <t>Look: Calm teal</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
-          <t>As Sunita, look for a Look/theme setting.</t>
+          <t>Same pages as above.</t>
         </is>
       </c>
       <c r="G107" s="5" t="inlineStr"/>
       <c r="H107" s="5" t="inlineStr">
         <is>
-          <t>Teachers cannot change the school look (no Look option).</t>
+          <t>Teal and white, simple. Everything readable, no overlap.</t>
         </is>
       </c>
       <c r="I107" s="5" t="inlineStr">
@@ -6388,7 +6392,7 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>LK-11</t>
+          <t>LK-09</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
@@ -6398,33 +6402,33 @@
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>Phone in dark mode</t>
+          <t>Look: Easy to read</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>Turn on Dark mode in the phone settings. Open the app.</t>
+          <t>Same pages as above, also outside in sunlight if possible.</t>
         </is>
       </c>
       <c r="G108" s="5" t="inlineStr"/>
       <c r="H108" s="5" t="inlineStr">
         <is>
-          <t>The app stays light (no dark mode in any look).</t>
+          <t>Black on white, thick borders, bigger letters. Very easy to read.</t>
         </is>
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J108" s="5" t="inlineStr">
@@ -6439,7 +6443,7 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>LK-12</t>
+          <t>LK-10</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -6449,33 +6453,33 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>School settings → Look</t>
+          <t>More → Me</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>At the end of testing: choose "Signal Shala" → "Use for the whole school".</t>
+          <t>As Sunita, look for a Look/theme setting.</t>
         </is>
       </c>
       <c r="G109" s="5" t="inlineStr"/>
       <c r="H109" s="5" t="inlineStr">
         <is>
-          <t>The school is back on the Signal Shala look.</t>
+          <t>Teachers cannot change the school look (no Look option).</t>
         </is>
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J109" s="5" t="inlineStr">
@@ -6490,12 +6494,12 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>GN-01</t>
+          <t>LK-11</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Looks</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
@@ -6510,23 +6514,23 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>Every page</t>
+          <t>Phone in dark mode</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>Use a small phone (or the smallest screen you have). Open each page.</t>
+          <t>Turn on Dark mode in the phone settings. Open the app.</t>
         </is>
       </c>
       <c r="G110" s="5" t="inlineStr"/>
       <c r="H110" s="5" t="inlineStr">
         <is>
-          <t>No page scrolls sideways; text is not cut; buttons are big enough to tap with a thumb.</t>
+          <t>The app stays light (no dark mode in any look).</t>
         </is>
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J110" s="5" t="inlineStr">
@@ -6541,43 +6545,43 @@
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>GN-02</t>
+          <t>LK-12</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Looks</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Phone + Computer</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>Any page</t>
+          <t>School settings → Look</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>Turn the phone sideways (landscape) on Today and Take attendance.</t>
+          <t>At the end of testing: choose "Signal Shala" → "Use for the whole school".</t>
         </is>
       </c>
       <c r="G111" s="5" t="inlineStr"/>
       <c r="H111" s="5" t="inlineStr">
         <is>
-          <t>Pages still work and look fine.</t>
+          <t>The school is back on the Signal Shala look.</t>
         </is>
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J111" s="5" t="inlineStr">
@@ -6592,7 +6596,7 @@
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>GN-03</t>
+          <t>GN-01</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
@@ -6612,23 +6616,23 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t>Chrome menu → Install app / Add to Home screen</t>
+          <t>Every page</t>
         </is>
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
-          <t>Install the app and open it from the home screen.</t>
+          <t>Use a small phone (or the smallest screen you have). Open each page.</t>
         </is>
       </c>
       <c r="G112" s="5" t="inlineStr"/>
       <c r="H112" s="5" t="inlineStr">
         <is>
-          <t>Opens like an app (no browser address bar), with the Signal School icon.</t>
+          <t>No page scrolls sideways; text is not cut; buttons are big enough to tap with a thumb.</t>
         </is>
       </c>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J112" s="5" t="inlineStr">
@@ -6643,7 +6647,7 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>GN-04</t>
+          <t>GN-02</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -6663,18 +6667,18 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>? buttons</t>
+          <t>Any page</t>
         </is>
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>Tap the "?" on Today, Students, Syllabus, Academic years.</t>
+          <t>Turn the phone sideways (landscape) on Today and Take attendance.</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr"/>
       <c r="H113" s="5" t="inlineStr">
         <is>
-          <t>A short help text in simple words appears.</t>
+          <t>Pages still work and look fine.</t>
         </is>
       </c>
       <c r="I113" s="5" t="inlineStr">
@@ -6694,7 +6698,7 @@
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>GN-05</t>
+          <t>GN-03</t>
         </is>
       </c>
       <c r="B114" s="5" t="inlineStr">
@@ -6714,18 +6718,18 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>Language check (मराठी / ગુજરાતી)</t>
+          <t>Chrome menu → Install app / Add to Home screen</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
-          <t>Switch to मराठी and then ગુજરાતી. Open Today, Attendance, Students, a student, Me.</t>
+          <t>Install the app and open it from the home screen.</t>
         </is>
       </c>
       <c r="G114" s="5" t="inlineStr"/>
       <c r="H114" s="5" t="inlineStr">
         <is>
-          <t>All words in that language and easy to read. Write in Comments any English words left or wrong spellings.</t>
+          <t>Opens like an app (no browser address bar), with the Signal School icon.</t>
         </is>
       </c>
       <c r="I114" s="5" t="inlineStr">
@@ -6745,7 +6749,7 @@
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>GN-06</t>
+          <t>GN-04</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
@@ -6760,28 +6764,28 @@
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t>Phone + Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
-          <t>Phone Back button / browser Back</t>
+          <t>? buttons</t>
         </is>
       </c>
       <c r="F115" s="5" t="inlineStr">
         <is>
-          <t>Move through several pages and press Back.</t>
+          <t>Tap the "?" on Today, Students, Syllabus, Academic years.</t>
         </is>
       </c>
       <c r="G115" s="5" t="inlineStr"/>
       <c r="H115" s="5" t="inlineStr">
         <is>
-          <t>Back goes to the previous page every time (does not exit the app unexpectedly).</t>
+          <t>A short help text in simple words appears.</t>
         </is>
       </c>
       <c r="I115" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J115" s="5" t="inlineStr">
@@ -6796,7 +6800,7 @@
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>GN-07</t>
+          <t>GN-05</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
@@ -6811,23 +6815,23 @@
       </c>
       <c r="D116" s="5" t="inlineStr">
         <is>
-          <t>Computer</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t>Computer, big window</t>
+          <t>Language check (मराठी / ગુજરાતી)</t>
         </is>
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
-          <t>Open on a computer. Make the window narrow, then wide.</t>
+          <t>Switch to मराठी and then ગુજરાતી. Open Today, Attendance, Students, a student, Me.</t>
         </is>
       </c>
       <c r="G116" s="5" t="inlineStr"/>
       <c r="H116" s="5" t="inlineStr">
         <is>
-          <t>Wide: side menu with groups "Every day", "School setup", "Other". Narrow: bottom bar like the phone.</t>
+          <t>All words in that language and easy to read. Write in Comments any English words left or wrong spellings.</t>
         </is>
       </c>
       <c r="I116" s="5" t="inlineStr">
@@ -6847,7 +6851,7 @@
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>GN-08</t>
+          <t>GN-06</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
@@ -6867,23 +6871,23 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t>Slow internet</t>
+          <t>Phone Back button / browser Back</t>
         </is>
       </c>
       <c r="F117" s="5" t="inlineStr">
         <is>
-          <t>In Chrome, use a slow connection (or weak mobile signal). Open Today and Students.</t>
+          <t>Move through several pages and press Back.</t>
         </is>
       </c>
       <c r="G117" s="5" t="inlineStr"/>
       <c r="H117" s="5" t="inlineStr">
         <is>
-          <t>Pages show a loading state and then load; nothing breaks.</t>
+          <t>Back goes to the previous page every time (does not exit the app unexpectedly).</t>
         </is>
       </c>
       <c r="I117" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J117" s="5" t="inlineStr">
@@ -6895,9 +6899,111 @@
       <c r="L117" s="5" t="inlineStr"/>
       <c r="M117" s="5" t="inlineStr"/>
     </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>GN-07</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>Computer</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>Computer, big window</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>Open on a computer. Make the window narrow, then wide.</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr"/>
+      <c r="H118" s="5" t="inlineStr">
+        <is>
+          <t>Wide: side menu with groups "Every day", "School setup", "Other". Narrow: bottom bar like the phone.</t>
+        </is>
+      </c>
+      <c r="I118" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J118" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="K118" s="5" t="inlineStr"/>
+      <c r="L118" s="5" t="inlineStr"/>
+      <c r="M118" s="5" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>GN-08</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>Phone + Computer</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>Slow internet</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>In Chrome, use a slow connection (or weak mobile signal). Open Today and Students.</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr"/>
+      <c r="H119" s="5" t="inlineStr">
+        <is>
+          <t>Pages show a loading state and then load; nothing breaks.</t>
+        </is>
+      </c>
+      <c r="I119" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J119" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="K119" s="5" t="inlineStr"/>
+      <c r="L119" s="5" t="inlineStr"/>
+      <c r="M119" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M117"/>
-  <conditionalFormatting sqref="J2:J117">
+  <autoFilter ref="A1:M119"/>
+  <conditionalFormatting sqref="J2:J119">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J2="Pass"</formula>
     </cfRule>
@@ -6911,13 +7017,13 @@
       <formula>$J2="Skipped"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I117">
+  <conditionalFormatting sqref="I2:I119">
     <cfRule type="expression" priority="5" dxfId="4">
       <formula>$I2="High"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J2:J119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not run,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8408,27 +8514,27 @@
         </is>
       </c>
       <c r="B2" s="8">
-        <f>COUNTIF('Test cases'!$B$2:$B$117,"Login*")</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$119,"Login*")</f>
         <v/>
       </c>
       <c r="C2" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Login*",'Test cases'!$J$2:$J$117,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Login*",'Test cases'!$J$2:$J$119,"Pass")</f>
         <v/>
       </c>
       <c r="D2" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Login*",'Test cases'!$J$2:$J$117,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Login*",'Test cases'!$J$2:$J$119,"Fail")</f>
         <v/>
       </c>
       <c r="E2" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Login*",'Test cases'!$J$2:$J$117,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Login*",'Test cases'!$J$2:$J$119,"Blocked")</f>
         <v/>
       </c>
       <c r="F2" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Login*",'Test cases'!$J$2:$J$117,"Skipped")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Login*",'Test cases'!$J$2:$J$119,"Skipped")</f>
         <v/>
       </c>
       <c r="G2" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Login*",'Test cases'!$J$2:$J$117,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Login*",'Test cases'!$J$2:$J$119,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -8439,27 +8545,27 @@
         </is>
       </c>
       <c r="B3" s="8">
-        <f>COUNTIF('Test cases'!$B$2:$B$117,"Teacher*")</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$119,"Teacher*")</f>
         <v/>
       </c>
       <c r="C3" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Teacher*",'Test cases'!$J$2:$J$117,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Teacher*",'Test cases'!$J$2:$J$119,"Pass")</f>
         <v/>
       </c>
       <c r="D3" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Teacher*",'Test cases'!$J$2:$J$117,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Teacher*",'Test cases'!$J$2:$J$119,"Fail")</f>
         <v/>
       </c>
       <c r="E3" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Teacher*",'Test cases'!$J$2:$J$117,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Teacher*",'Test cases'!$J$2:$J$119,"Blocked")</f>
         <v/>
       </c>
       <c r="F3" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Teacher*",'Test cases'!$J$2:$J$117,"Skipped")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Teacher*",'Test cases'!$J$2:$J$119,"Skipped")</f>
         <v/>
       </c>
       <c r="G3" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Teacher*",'Test cases'!$J$2:$J$117,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Teacher*",'Test cases'!$J$2:$J$119,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -8470,27 +8576,27 @@
         </is>
       </c>
       <c r="B4" s="8">
-        <f>COUNTIF('Test cases'!$B$2:$B$117,"Office clerk*")</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$119,"Office clerk*")</f>
         <v/>
       </c>
       <c r="C4" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Office clerk*",'Test cases'!$J$2:$J$117,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Office clerk*",'Test cases'!$J$2:$J$119,"Pass")</f>
         <v/>
       </c>
       <c r="D4" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Office clerk*",'Test cases'!$J$2:$J$117,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Office clerk*",'Test cases'!$J$2:$J$119,"Fail")</f>
         <v/>
       </c>
       <c r="E4" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Office clerk*",'Test cases'!$J$2:$J$117,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Office clerk*",'Test cases'!$J$2:$J$119,"Blocked")</f>
         <v/>
       </c>
       <c r="F4" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Office clerk*",'Test cases'!$J$2:$J$117,"Skipped")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Office clerk*",'Test cases'!$J$2:$J$119,"Skipped")</f>
         <v/>
       </c>
       <c r="G4" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Office clerk*",'Test cases'!$J$2:$J$117,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Office clerk*",'Test cases'!$J$2:$J$119,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -8501,27 +8607,27 @@
         </is>
       </c>
       <c r="B5" s="8">
-        <f>COUNTIF('Test cases'!$B$2:$B$117,"Principal*")</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$119,"Principal*")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Principal*",'Test cases'!$J$2:$J$117,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Principal*",'Test cases'!$J$2:$J$119,"Pass")</f>
         <v/>
       </c>
       <c r="D5" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Principal*",'Test cases'!$J$2:$J$117,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Principal*",'Test cases'!$J$2:$J$119,"Fail")</f>
         <v/>
       </c>
       <c r="E5" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Principal*",'Test cases'!$J$2:$J$117,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Principal*",'Test cases'!$J$2:$J$119,"Blocked")</f>
         <v/>
       </c>
       <c r="F5" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Principal*",'Test cases'!$J$2:$J$117,"Skipped")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Principal*",'Test cases'!$J$2:$J$119,"Skipped")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Principal*",'Test cases'!$J$2:$J$117,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Principal*",'Test cases'!$J$2:$J$119,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -8532,27 +8638,27 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>COUNTIF('Test cases'!$B$2:$B$117,"Trust owner*")</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$119,"Trust owner*")</f>
         <v/>
       </c>
       <c r="C6" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Trust owner*",'Test cases'!$J$2:$J$117,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Trust owner*",'Test cases'!$J$2:$J$119,"Pass")</f>
         <v/>
       </c>
       <c r="D6" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Trust owner*",'Test cases'!$J$2:$J$117,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Trust owner*",'Test cases'!$J$2:$J$119,"Fail")</f>
         <v/>
       </c>
       <c r="E6" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Trust owner*",'Test cases'!$J$2:$J$117,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Trust owner*",'Test cases'!$J$2:$J$119,"Blocked")</f>
         <v/>
       </c>
       <c r="F6" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Trust owner*",'Test cases'!$J$2:$J$117,"Skipped")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Trust owner*",'Test cases'!$J$2:$J$119,"Skipped")</f>
         <v/>
       </c>
       <c r="G6" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Trust owner*",'Test cases'!$J$2:$J$117,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Trust owner*",'Test cases'!$J$2:$J$119,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -8563,27 +8669,27 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>COUNTIF('Test cases'!$B$2:$B$117,"Looks*")</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$119,"Looks*")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Looks*",'Test cases'!$J$2:$J$117,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Looks*",'Test cases'!$J$2:$J$119,"Pass")</f>
         <v/>
       </c>
       <c r="D7" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Looks*",'Test cases'!$J$2:$J$117,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Looks*",'Test cases'!$J$2:$J$119,"Fail")</f>
         <v/>
       </c>
       <c r="E7" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Looks*",'Test cases'!$J$2:$J$117,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Looks*",'Test cases'!$J$2:$J$119,"Blocked")</f>
         <v/>
       </c>
       <c r="F7" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Looks*",'Test cases'!$J$2:$J$117,"Skipped")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Looks*",'Test cases'!$J$2:$J$119,"Skipped")</f>
         <v/>
       </c>
       <c r="G7" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"Looks*",'Test cases'!$J$2:$J$117,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"Looks*",'Test cases'!$J$2:$J$119,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -8594,27 +8700,27 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>COUNTIF('Test cases'!$B$2:$B$117,"General*")</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$119,"General*")</f>
         <v/>
       </c>
       <c r="C8" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"General*",'Test cases'!$J$2:$J$117,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"General*",'Test cases'!$J$2:$J$119,"Pass")</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"General*",'Test cases'!$J$2:$J$117,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"General*",'Test cases'!$J$2:$J$119,"Fail")</f>
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"General*",'Test cases'!$J$2:$J$117,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"General*",'Test cases'!$J$2:$J$119,"Blocked")</f>
         <v/>
       </c>
       <c r="F8" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"General*",'Test cases'!$J$2:$J$117,"Skipped")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"General*",'Test cases'!$J$2:$J$119,"Skipped")</f>
         <v/>
       </c>
       <c r="G8" s="8">
-        <f>COUNTIFS('Test cases'!$B$2:$B$117,"General*",'Test cases'!$J$2:$J$117,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$119,"General*",'Test cases'!$J$2:$J$119,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -8625,27 +8731,27 @@
         </is>
       </c>
       <c r="B9" s="9">
-        <f>COUNTA('Test cases'!$J$2:$J$117)</f>
+        <f>COUNTA('Test cases'!$J$2:$J$119)</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>COUNTIF('Test cases'!$J$2:$J$117,"Pass")</f>
+        <f>COUNTIF('Test cases'!$J$2:$J$119,"Pass")</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>COUNTIF('Test cases'!$J$2:$J$117,"Fail")</f>
+        <f>COUNTIF('Test cases'!$J$2:$J$119,"Fail")</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>COUNTIF('Test cases'!$J$2:$J$117,"Blocked")</f>
+        <f>COUNTIF('Test cases'!$J$2:$J$119,"Blocked")</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>COUNTIF('Test cases'!$J$2:$J$117,"Skipped")</f>
+        <f>COUNTIF('Test cases'!$J$2:$J$119,"Skipped")</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>COUNTIF('Test cases'!$J$2:$J$117,"Not run")</f>
+        <f>COUNTIF('Test cases'!$J$2:$J$119,"Not run")</f>
         <v/>
       </c>
     </row>

</xml_diff>